<commit_message>
Donovan Part 2 bby
Finished up my individual and added my regulatory comparison, kind of following Ethan's Style. Waiting on everyone to finish their portions of the regulatory comparison, to get a matrix put in place for us to finish step 6.
</commit_message>
<xml_diff>
--- a/analysis/manogue/privacy_policy_summary.xlsx
+++ b/analysis/manogue/privacy_policy_summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Donovan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bd449e93427ae247/Documents/GitHub/DATA6550-Privacy-Audit/analysis/manogue/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3111F94-12D0-4BDA-B026-2813320123E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{F3111F94-12D0-4BDA-B026-2813320123E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F086B9E-5A9D-435D-96A8-CCEC00DB77E1}"/>
   <bookViews>
-    <workbookView xWindow="2520" yWindow="3075" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37620" yWindow="945" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chase Bank" sheetId="1" r:id="rId1"/>
@@ -528,13 +528,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{59CF5FBF-3674-480B-96B0-6B79FAB4D585}" name="Table2" displayName="Table2" ref="A1:D6" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{59CF5FBF-3674-480B-96B0-6B79FAB4D585}" name="Table2" displayName="Table2" ref="A1:D6" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="A1:D6" xr:uid="{59CF5FBF-3674-480B-96B0-6B79FAB4D585}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{16C1E5A1-C6B7-43D4-B17B-F74A7DCC043C}" name="Category" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{B139156F-795D-4832-89D7-EA619B1C5F51}" name="Rating (0-5)" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{815AE397-53D0-4095-8791-C9E748EC51DF}" name="Category Label" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{0AC56EA1-A0A5-40C5-879F-B727192CED40}" name="Key Insight" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{16C1E5A1-C6B7-43D4-B17B-F74A7DCC043C}" name="Category" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{B139156F-795D-4832-89D7-EA619B1C5F51}" name="Rating (0-5)" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{815AE397-53D0-4095-8791-C9E748EC51DF}" name="Category Label" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{0AC56EA1-A0A5-40C5-879F-B727192CED40}" name="Key Insight" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -828,10 +828,10 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="95.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="118.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">

</xml_diff>